<commit_message>
add and update template sertifikat kalibrasi
</commit_message>
<xml_diff>
--- a/public/assets/templates/template_kalibrasi_pressure_sertifikat.xlsx
+++ b/public/assets/templates/template_kalibrasi_pressure_sertifikat.xlsx
@@ -8,16 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\pt_bas\Engineering\public\assets\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5FF4DC4-D8E1-47B3-A09F-17F8FE3DE5CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0738FBD8-8065-44BF-A917-2954EBC440FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10560" xr2:uid="{D57B88DC-6A9D-42A6-BE16-0F559C48DA93}"/>
   </bookViews>
   <sheets>
     <sheet name="Sertifikat" sheetId="1" r:id="rId1"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId2"/>
-  </externalReferences>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">Sertifikat!$B$2:$AJ$70</definedName>
   </definedNames>
@@ -889,20 +886,20 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1060,17 +1057,17 @@
           </c:marker>
           <c:val>
             <c:numRef>
-              <c:f>Sertifikat!$H$26:$H$35</c:f>
+              <c:f>Sertifikat!$H$26:$H$32</c:f>
               <c:numCache>
                 <c:formatCode>0.0_ </c:formatCode>
-                <c:ptCount val="10"/>
+                <c:ptCount val="7"/>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-1680-4EB8-B1FC-AE50047EA0ED}"/>
+              <c16:uniqueId val="{00000000-6C72-4356-A7AC-15A840331872}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1109,17 +1106,17 @@
           </c:marker>
           <c:val>
             <c:numRef>
-              <c:f>Sertifikat!$L$26:$L$35</c:f>
+              <c:f>Sertifikat!$L$26:$L$32</c:f>
               <c:numCache>
                 <c:formatCode>0.0_ </c:formatCode>
-                <c:ptCount val="10"/>
+                <c:ptCount val="7"/>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-1680-4EB8-B1FC-AE50047EA0ED}"/>
+              <c16:uniqueId val="{00000001-6C72-4356-A7AC-15A840331872}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1158,17 +1155,17 @@
           </c:marker>
           <c:val>
             <c:numRef>
-              <c:f>Sertifikat!$O$26:$O$35</c:f>
+              <c:f>Sertifikat!$O$26:$O$32</c:f>
               <c:numCache>
                 <c:formatCode>0.0_ </c:formatCode>
-                <c:ptCount val="10"/>
+                <c:ptCount val="7"/>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-1680-4EB8-B1FC-AE50047EA0ED}"/>
+              <c16:uniqueId val="{00000002-6C72-4356-A7AC-15A840331872}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1205,17 +1202,17 @@
           </c:marker>
           <c:val>
             <c:numRef>
-              <c:f>Sertifikat!$R$26:$R$35</c:f>
+              <c:f>Sertifikat!$R$26:$R$32</c:f>
               <c:numCache>
                 <c:formatCode>0.0_ </c:formatCode>
-                <c:ptCount val="10"/>
+                <c:ptCount val="7"/>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-1680-4EB8-B1FC-AE50047EA0ED}"/>
+              <c16:uniqueId val="{00000003-6C72-4356-A7AC-15A840331872}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1256,17 +1253,17 @@
           </c:marker>
           <c:val>
             <c:numRef>
-              <c:f>Sertifikat!$U$26:$U$35</c:f>
+              <c:f>Sertifikat!$U$26:$U$32</c:f>
               <c:numCache>
                 <c:formatCode>0.0_ </c:formatCode>
-                <c:ptCount val="10"/>
+                <c:ptCount val="7"/>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-1680-4EB8-B1FC-AE50047EA0ED}"/>
+              <c16:uniqueId val="{00000004-6C72-4356-A7AC-15A840331872}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1280,11 +1277,11 @@
         </c:dLbls>
         <c:marker val="1"/>
         <c:smooth val="0"/>
-        <c:axId val="283134335"/>
+        <c:axId val="936390815"/>
         <c:axId val="1"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="283134335"/>
+        <c:axId val="936390815"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1382,7 +1379,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="283134335"/>
+        <c:crossAx val="936390815"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="1"/>
@@ -1555,22 +1552,22 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>260350</xdr:colOff>
+      <xdr:colOff>266700</xdr:colOff>
       <xdr:row>40</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>31750</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>30</xdr:col>
-      <xdr:colOff>150533</xdr:colOff>
+      <xdr:colOff>76200</xdr:colOff>
       <xdr:row>48</xdr:row>
-      <xdr:rowOff>201706</xdr:rowOff>
+      <xdr:rowOff>203200</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="4" name="Chart 3">
+        <xdr:cNvPr id="3" name="Chart 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1E41C6A1-CE7B-4687-9CCC-CB76351181A2}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2C1A6C03-80B8-4C89-8DA4-EC7C8F19F8AC}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1591,128 +1588,6 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <sheetNames>
-      <sheetName val="Hitung Tekanan Naik"/>
-      <sheetName val="Hitung Tekanan Turun"/>
-      <sheetName val="Hitung U Gabungan"/>
-      <sheetName val="Sertifikat "/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3">
-        <row r="26">
-          <cell r="H26">
-            <v>0</v>
-          </cell>
-          <cell r="L26">
-            <v>0</v>
-          </cell>
-          <cell r="O26">
-            <v>0</v>
-          </cell>
-          <cell r="R26">
-            <v>0</v>
-          </cell>
-          <cell r="U26">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="27">
-          <cell r="H27">
-            <v>0.98066500000000001</v>
-          </cell>
-          <cell r="L27">
-            <v>0.98066500000000001</v>
-          </cell>
-          <cell r="O27">
-            <v>0.98066500000000001</v>
-          </cell>
-          <cell r="R27">
-            <v>1.2</v>
-          </cell>
-          <cell r="U27">
-            <v>1.2</v>
-          </cell>
-        </row>
-        <row r="28">
-          <cell r="H28">
-            <v>1.96133</v>
-          </cell>
-          <cell r="L28">
-            <v>1.96133</v>
-          </cell>
-          <cell r="O28">
-            <v>1.96133</v>
-          </cell>
-          <cell r="R28">
-            <v>2.1</v>
-          </cell>
-          <cell r="U28">
-            <v>2.1</v>
-          </cell>
-        </row>
-        <row r="29">
-          <cell r="H29">
-            <v>3</v>
-          </cell>
-          <cell r="L29">
-            <v>3</v>
-          </cell>
-          <cell r="O29">
-            <v>3</v>
-          </cell>
-          <cell r="R29">
-            <v>3.1</v>
-          </cell>
-          <cell r="U29">
-            <v>3.1</v>
-          </cell>
-        </row>
-        <row r="30">
-          <cell r="H30">
-            <v>4</v>
-          </cell>
-          <cell r="L30">
-            <v>4</v>
-          </cell>
-          <cell r="O30">
-            <v>4</v>
-          </cell>
-          <cell r="R30">
-            <v>4.0999999999999996</v>
-          </cell>
-          <cell r="U30">
-            <v>4.0999999999999996</v>
-          </cell>
-        </row>
-        <row r="31">
-          <cell r="H31">
-            <v>5</v>
-          </cell>
-          <cell r="L31">
-            <v>5</v>
-          </cell>
-          <cell r="O31">
-            <v>5</v>
-          </cell>
-          <cell r="R31">
-            <v>5.0999999999999996</v>
-          </cell>
-          <cell r="U31">
-            <v>5.0999999999999996</v>
-          </cell>
-        </row>
-      </sheetData>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3096,11 +2971,11 @@
       <c r="I25" s="71"/>
       <c r="J25" s="71"/>
       <c r="K25" s="72"/>
-      <c r="L25" s="73" t="s">
+      <c r="L25" s="77" t="s">
         <v>27</v>
       </c>
-      <c r="M25" s="73"/>
-      <c r="N25" s="73"/>
+      <c r="M25" s="77"/>
+      <c r="N25" s="77"/>
       <c r="O25" s="55" t="s">
         <v>27</v>
       </c>
@@ -3149,30 +3024,30 @@
       <c r="I26" s="66"/>
       <c r="J26" s="66"/>
       <c r="K26" s="66"/>
-      <c r="L26" s="74"/>
-      <c r="M26" s="74"/>
-      <c r="N26" s="74"/>
-      <c r="O26" s="74"/>
-      <c r="P26" s="74"/>
-      <c r="Q26" s="74"/>
-      <c r="R26" s="74"/>
-      <c r="S26" s="74"/>
-      <c r="T26" s="74"/>
-      <c r="U26" s="74"/>
-      <c r="V26" s="74"/>
-      <c r="W26" s="74"/>
-      <c r="X26" s="74"/>
-      <c r="Y26" s="74"/>
-      <c r="Z26" s="74"/>
-      <c r="AA26" s="74"/>
-      <c r="AB26" s="74"/>
-      <c r="AC26" s="74"/>
-      <c r="AD26" s="75"/>
-      <c r="AE26" s="76"/>
-      <c r="AF26" s="76"/>
-      <c r="AG26" s="76"/>
-      <c r="AH26" s="76"/>
-      <c r="AI26" s="77"/>
+      <c r="L26" s="73"/>
+      <c r="M26" s="73"/>
+      <c r="N26" s="73"/>
+      <c r="O26" s="73"/>
+      <c r="P26" s="73"/>
+      <c r="Q26" s="73"/>
+      <c r="R26" s="73"/>
+      <c r="S26" s="73"/>
+      <c r="T26" s="73"/>
+      <c r="U26" s="73"/>
+      <c r="V26" s="73"/>
+      <c r="W26" s="73"/>
+      <c r="X26" s="73"/>
+      <c r="Y26" s="73"/>
+      <c r="Z26" s="73"/>
+      <c r="AA26" s="73"/>
+      <c r="AB26" s="73"/>
+      <c r="AC26" s="73"/>
+      <c r="AD26" s="74"/>
+      <c r="AE26" s="75"/>
+      <c r="AF26" s="75"/>
+      <c r="AG26" s="75"/>
+      <c r="AH26" s="75"/>
+      <c r="AI26" s="76"/>
       <c r="AJ26" s="8"/>
     </row>
     <row r="27" spans="2:36" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -3184,34 +3059,34 @@
       <c r="E27" s="66"/>
       <c r="F27" s="66"/>
       <c r="G27" s="66"/>
-      <c r="H27" s="74"/>
-      <c r="I27" s="74"/>
-      <c r="J27" s="74"/>
-      <c r="K27" s="74"/>
-      <c r="L27" s="74"/>
-      <c r="M27" s="74"/>
-      <c r="N27" s="74"/>
-      <c r="O27" s="74"/>
-      <c r="P27" s="74"/>
-      <c r="Q27" s="74"/>
-      <c r="R27" s="74"/>
-      <c r="S27" s="74"/>
-      <c r="T27" s="74"/>
-      <c r="U27" s="74"/>
-      <c r="V27" s="74"/>
-      <c r="W27" s="74"/>
-      <c r="X27" s="74"/>
-      <c r="Y27" s="74"/>
-      <c r="Z27" s="74"/>
-      <c r="AA27" s="74"/>
-      <c r="AB27" s="74"/>
-      <c r="AC27" s="74"/>
-      <c r="AD27" s="75"/>
-      <c r="AE27" s="76"/>
-      <c r="AF27" s="76"/>
-      <c r="AG27" s="76"/>
-      <c r="AH27" s="76"/>
-      <c r="AI27" s="77"/>
+      <c r="H27" s="73"/>
+      <c r="I27" s="73"/>
+      <c r="J27" s="73"/>
+      <c r="K27" s="73"/>
+      <c r="L27" s="73"/>
+      <c r="M27" s="73"/>
+      <c r="N27" s="73"/>
+      <c r="O27" s="73"/>
+      <c r="P27" s="73"/>
+      <c r="Q27" s="73"/>
+      <c r="R27" s="73"/>
+      <c r="S27" s="73"/>
+      <c r="T27" s="73"/>
+      <c r="U27" s="73"/>
+      <c r="V27" s="73"/>
+      <c r="W27" s="73"/>
+      <c r="X27" s="73"/>
+      <c r="Y27" s="73"/>
+      <c r="Z27" s="73"/>
+      <c r="AA27" s="73"/>
+      <c r="AB27" s="73"/>
+      <c r="AC27" s="73"/>
+      <c r="AD27" s="74"/>
+      <c r="AE27" s="75"/>
+      <c r="AF27" s="75"/>
+      <c r="AG27" s="75"/>
+      <c r="AH27" s="75"/>
+      <c r="AI27" s="76"/>
       <c r="AJ27" s="8"/>
     </row>
     <row r="28" spans="2:36" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -3223,34 +3098,34 @@
       <c r="E28" s="66"/>
       <c r="F28" s="66"/>
       <c r="G28" s="66"/>
-      <c r="H28" s="74"/>
-      <c r="I28" s="74"/>
-      <c r="J28" s="74"/>
-      <c r="K28" s="74"/>
-      <c r="L28" s="74"/>
-      <c r="M28" s="74"/>
-      <c r="N28" s="74"/>
-      <c r="O28" s="74"/>
-      <c r="P28" s="74"/>
-      <c r="Q28" s="74"/>
-      <c r="R28" s="74"/>
-      <c r="S28" s="74"/>
-      <c r="T28" s="74"/>
-      <c r="U28" s="74"/>
-      <c r="V28" s="74"/>
-      <c r="W28" s="74"/>
-      <c r="X28" s="74"/>
-      <c r="Y28" s="74"/>
-      <c r="Z28" s="74"/>
-      <c r="AA28" s="74"/>
-      <c r="AB28" s="74"/>
-      <c r="AC28" s="74"/>
-      <c r="AD28" s="75"/>
-      <c r="AE28" s="76"/>
-      <c r="AF28" s="76"/>
-      <c r="AG28" s="76"/>
-      <c r="AH28" s="76"/>
-      <c r="AI28" s="77"/>
+      <c r="H28" s="73"/>
+      <c r="I28" s="73"/>
+      <c r="J28" s="73"/>
+      <c r="K28" s="73"/>
+      <c r="L28" s="73"/>
+      <c r="M28" s="73"/>
+      <c r="N28" s="73"/>
+      <c r="O28" s="73"/>
+      <c r="P28" s="73"/>
+      <c r="Q28" s="73"/>
+      <c r="R28" s="73"/>
+      <c r="S28" s="73"/>
+      <c r="T28" s="73"/>
+      <c r="U28" s="73"/>
+      <c r="V28" s="73"/>
+      <c r="W28" s="73"/>
+      <c r="X28" s="73"/>
+      <c r="Y28" s="73"/>
+      <c r="Z28" s="73"/>
+      <c r="AA28" s="73"/>
+      <c r="AB28" s="73"/>
+      <c r="AC28" s="73"/>
+      <c r="AD28" s="74"/>
+      <c r="AE28" s="75"/>
+      <c r="AF28" s="75"/>
+      <c r="AG28" s="75"/>
+      <c r="AH28" s="75"/>
+      <c r="AI28" s="76"/>
       <c r="AJ28" s="19"/>
     </row>
     <row r="29" spans="2:36" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -3262,34 +3137,34 @@
       <c r="E29" s="66"/>
       <c r="F29" s="66"/>
       <c r="G29" s="66"/>
-      <c r="H29" s="74"/>
-      <c r="I29" s="74"/>
-      <c r="J29" s="74"/>
-      <c r="K29" s="74"/>
-      <c r="L29" s="74"/>
-      <c r="M29" s="74"/>
-      <c r="N29" s="74"/>
-      <c r="O29" s="74"/>
-      <c r="P29" s="74"/>
-      <c r="Q29" s="74"/>
-      <c r="R29" s="74"/>
-      <c r="S29" s="74"/>
-      <c r="T29" s="74"/>
-      <c r="U29" s="74"/>
-      <c r="V29" s="74"/>
-      <c r="W29" s="74"/>
-      <c r="X29" s="74"/>
-      <c r="Y29" s="74"/>
-      <c r="Z29" s="74"/>
-      <c r="AA29" s="74"/>
-      <c r="AB29" s="74"/>
-      <c r="AC29" s="74"/>
-      <c r="AD29" s="75"/>
-      <c r="AE29" s="76"/>
-      <c r="AF29" s="76"/>
-      <c r="AG29" s="76"/>
-      <c r="AH29" s="76"/>
-      <c r="AI29" s="77"/>
+      <c r="H29" s="73"/>
+      <c r="I29" s="73"/>
+      <c r="J29" s="73"/>
+      <c r="K29" s="73"/>
+      <c r="L29" s="73"/>
+      <c r="M29" s="73"/>
+      <c r="N29" s="73"/>
+      <c r="O29" s="73"/>
+      <c r="P29" s="73"/>
+      <c r="Q29" s="73"/>
+      <c r="R29" s="73"/>
+      <c r="S29" s="73"/>
+      <c r="T29" s="73"/>
+      <c r="U29" s="73"/>
+      <c r="V29" s="73"/>
+      <c r="W29" s="73"/>
+      <c r="X29" s="73"/>
+      <c r="Y29" s="73"/>
+      <c r="Z29" s="73"/>
+      <c r="AA29" s="73"/>
+      <c r="AB29" s="73"/>
+      <c r="AC29" s="73"/>
+      <c r="AD29" s="74"/>
+      <c r="AE29" s="75"/>
+      <c r="AF29" s="75"/>
+      <c r="AG29" s="75"/>
+      <c r="AH29" s="75"/>
+      <c r="AI29" s="76"/>
       <c r="AJ29" s="19"/>
     </row>
     <row r="30" spans="2:36" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -3301,34 +3176,34 @@
       <c r="E30" s="66"/>
       <c r="F30" s="66"/>
       <c r="G30" s="66"/>
-      <c r="H30" s="74"/>
-      <c r="I30" s="74"/>
-      <c r="J30" s="74"/>
-      <c r="K30" s="74"/>
-      <c r="L30" s="74"/>
-      <c r="M30" s="74"/>
-      <c r="N30" s="74"/>
-      <c r="O30" s="74"/>
-      <c r="P30" s="74"/>
-      <c r="Q30" s="74"/>
-      <c r="R30" s="74"/>
-      <c r="S30" s="74"/>
-      <c r="T30" s="74"/>
-      <c r="U30" s="74"/>
-      <c r="V30" s="74"/>
-      <c r="W30" s="74"/>
-      <c r="X30" s="74"/>
-      <c r="Y30" s="74"/>
-      <c r="Z30" s="74"/>
+      <c r="H30" s="73"/>
+      <c r="I30" s="73"/>
+      <c r="J30" s="73"/>
+      <c r="K30" s="73"/>
+      <c r="L30" s="73"/>
+      <c r="M30" s="73"/>
+      <c r="N30" s="73"/>
+      <c r="O30" s="73"/>
+      <c r="P30" s="73"/>
+      <c r="Q30" s="73"/>
+      <c r="R30" s="73"/>
+      <c r="S30" s="73"/>
+      <c r="T30" s="73"/>
+      <c r="U30" s="73"/>
+      <c r="V30" s="73"/>
+      <c r="W30" s="73"/>
+      <c r="X30" s="73"/>
+      <c r="Y30" s="73"/>
+      <c r="Z30" s="73"/>
       <c r="AA30" s="78"/>
       <c r="AB30" s="78"/>
       <c r="AC30" s="78"/>
-      <c r="AD30" s="75"/>
-      <c r="AE30" s="76"/>
-      <c r="AF30" s="76"/>
-      <c r="AG30" s="76"/>
-      <c r="AH30" s="76"/>
-      <c r="AI30" s="77"/>
+      <c r="AD30" s="74"/>
+      <c r="AE30" s="75"/>
+      <c r="AF30" s="75"/>
+      <c r="AG30" s="75"/>
+      <c r="AH30" s="75"/>
+      <c r="AI30" s="76"/>
       <c r="AJ30" s="19"/>
     </row>
     <row r="31" spans="2:36" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -3340,34 +3215,34 @@
       <c r="E31" s="66"/>
       <c r="F31" s="66"/>
       <c r="G31" s="66"/>
-      <c r="H31" s="74"/>
-      <c r="I31" s="74"/>
-      <c r="J31" s="74"/>
-      <c r="K31" s="74"/>
-      <c r="L31" s="74"/>
-      <c r="M31" s="74"/>
-      <c r="N31" s="74"/>
-      <c r="O31" s="74"/>
-      <c r="P31" s="74"/>
-      <c r="Q31" s="74"/>
-      <c r="R31" s="74"/>
-      <c r="S31" s="74"/>
-      <c r="T31" s="74"/>
-      <c r="U31" s="74"/>
-      <c r="V31" s="74"/>
-      <c r="W31" s="74"/>
-      <c r="X31" s="74"/>
-      <c r="Y31" s="74"/>
-      <c r="Z31" s="74"/>
-      <c r="AA31" s="74"/>
-      <c r="AB31" s="74"/>
-      <c r="AC31" s="74"/>
-      <c r="AD31" s="75"/>
-      <c r="AE31" s="76"/>
-      <c r="AF31" s="76"/>
-      <c r="AG31" s="76"/>
-      <c r="AH31" s="76"/>
-      <c r="AI31" s="77"/>
+      <c r="H31" s="73"/>
+      <c r="I31" s="73"/>
+      <c r="J31" s="73"/>
+      <c r="K31" s="73"/>
+      <c r="L31" s="73"/>
+      <c r="M31" s="73"/>
+      <c r="N31" s="73"/>
+      <c r="O31" s="73"/>
+      <c r="P31" s="73"/>
+      <c r="Q31" s="73"/>
+      <c r="R31" s="73"/>
+      <c r="S31" s="73"/>
+      <c r="T31" s="73"/>
+      <c r="U31" s="73"/>
+      <c r="V31" s="73"/>
+      <c r="W31" s="73"/>
+      <c r="X31" s="73"/>
+      <c r="Y31" s="73"/>
+      <c r="Z31" s="73"/>
+      <c r="AA31" s="73"/>
+      <c r="AB31" s="73"/>
+      <c r="AC31" s="73"/>
+      <c r="AD31" s="74"/>
+      <c r="AE31" s="75"/>
+      <c r="AF31" s="75"/>
+      <c r="AG31" s="75"/>
+      <c r="AH31" s="75"/>
+      <c r="AI31" s="76"/>
       <c r="AJ31" s="19"/>
     </row>
     <row r="32" spans="2:36" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -3379,34 +3254,34 @@
       <c r="E32" s="66"/>
       <c r="F32" s="66"/>
       <c r="G32" s="66"/>
-      <c r="H32" s="74"/>
-      <c r="I32" s="74"/>
-      <c r="J32" s="74"/>
-      <c r="K32" s="74"/>
-      <c r="L32" s="74"/>
-      <c r="M32" s="74"/>
-      <c r="N32" s="74"/>
-      <c r="O32" s="74"/>
-      <c r="P32" s="74"/>
-      <c r="Q32" s="74"/>
-      <c r="R32" s="74"/>
-      <c r="S32" s="74"/>
-      <c r="T32" s="74"/>
-      <c r="U32" s="74"/>
-      <c r="V32" s="74"/>
-      <c r="W32" s="74"/>
-      <c r="X32" s="74"/>
-      <c r="Y32" s="74"/>
-      <c r="Z32" s="74"/>
-      <c r="AA32" s="74"/>
-      <c r="AB32" s="74"/>
-      <c r="AC32" s="74"/>
-      <c r="AD32" s="75"/>
-      <c r="AE32" s="76"/>
-      <c r="AF32" s="76"/>
-      <c r="AG32" s="76"/>
-      <c r="AH32" s="76"/>
-      <c r="AI32" s="77"/>
+      <c r="H32" s="73"/>
+      <c r="I32" s="73"/>
+      <c r="J32" s="73"/>
+      <c r="K32" s="73"/>
+      <c r="L32" s="73"/>
+      <c r="M32" s="73"/>
+      <c r="N32" s="73"/>
+      <c r="O32" s="73"/>
+      <c r="P32" s="73"/>
+      <c r="Q32" s="73"/>
+      <c r="R32" s="73"/>
+      <c r="S32" s="73"/>
+      <c r="T32" s="73"/>
+      <c r="U32" s="73"/>
+      <c r="V32" s="73"/>
+      <c r="W32" s="73"/>
+      <c r="X32" s="73"/>
+      <c r="Y32" s="73"/>
+      <c r="Z32" s="73"/>
+      <c r="AA32" s="73"/>
+      <c r="AB32" s="73"/>
+      <c r="AC32" s="73"/>
+      <c r="AD32" s="74"/>
+      <c r="AE32" s="75"/>
+      <c r="AF32" s="75"/>
+      <c r="AG32" s="75"/>
+      <c r="AH32" s="75"/>
+      <c r="AI32" s="76"/>
       <c r="AJ32" s="8"/>
     </row>
     <row r="33" spans="2:36" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -3428,24 +3303,24 @@
       <c r="O33" s="66"/>
       <c r="P33" s="66"/>
       <c r="Q33" s="66"/>
-      <c r="R33" s="74"/>
-      <c r="S33" s="74"/>
-      <c r="T33" s="74"/>
-      <c r="U33" s="74"/>
-      <c r="V33" s="74"/>
-      <c r="W33" s="74"/>
-      <c r="X33" s="74"/>
-      <c r="Y33" s="74"/>
-      <c r="Z33" s="74"/>
-      <c r="AA33" s="74"/>
-      <c r="AB33" s="74"/>
-      <c r="AC33" s="74"/>
-      <c r="AD33" s="75"/>
-      <c r="AE33" s="76"/>
-      <c r="AF33" s="76"/>
-      <c r="AG33" s="76"/>
-      <c r="AH33" s="76"/>
-      <c r="AI33" s="77"/>
+      <c r="R33" s="73"/>
+      <c r="S33" s="73"/>
+      <c r="T33" s="73"/>
+      <c r="U33" s="73"/>
+      <c r="V33" s="73"/>
+      <c r="W33" s="73"/>
+      <c r="X33" s="73"/>
+      <c r="Y33" s="73"/>
+      <c r="Z33" s="73"/>
+      <c r="AA33" s="73"/>
+      <c r="AB33" s="73"/>
+      <c r="AC33" s="73"/>
+      <c r="AD33" s="74"/>
+      <c r="AE33" s="75"/>
+      <c r="AF33" s="75"/>
+      <c r="AG33" s="75"/>
+      <c r="AH33" s="75"/>
+      <c r="AI33" s="76"/>
       <c r="AJ33" s="8"/>
     </row>
     <row r="34" spans="2:36" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -3467,24 +3342,24 @@
       <c r="O34" s="66"/>
       <c r="P34" s="66"/>
       <c r="Q34" s="66"/>
-      <c r="R34" s="74"/>
-      <c r="S34" s="74"/>
-      <c r="T34" s="74"/>
-      <c r="U34" s="74"/>
-      <c r="V34" s="74"/>
-      <c r="W34" s="74"/>
-      <c r="X34" s="74"/>
-      <c r="Y34" s="74"/>
-      <c r="Z34" s="74"/>
-      <c r="AA34" s="74"/>
-      <c r="AB34" s="74"/>
-      <c r="AC34" s="74"/>
-      <c r="AD34" s="75"/>
-      <c r="AE34" s="76"/>
-      <c r="AF34" s="76"/>
-      <c r="AG34" s="76"/>
-      <c r="AH34" s="76"/>
-      <c r="AI34" s="77"/>
+      <c r="R34" s="73"/>
+      <c r="S34" s="73"/>
+      <c r="T34" s="73"/>
+      <c r="U34" s="73"/>
+      <c r="V34" s="73"/>
+      <c r="W34" s="73"/>
+      <c r="X34" s="73"/>
+      <c r="Y34" s="73"/>
+      <c r="Z34" s="73"/>
+      <c r="AA34" s="73"/>
+      <c r="AB34" s="73"/>
+      <c r="AC34" s="73"/>
+      <c r="AD34" s="74"/>
+      <c r="AE34" s="75"/>
+      <c r="AF34" s="75"/>
+      <c r="AG34" s="75"/>
+      <c r="AH34" s="75"/>
+      <c r="AI34" s="76"/>
       <c r="AJ34" s="8"/>
     </row>
     <row r="35" spans="2:36" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -3506,24 +3381,24 @@
       <c r="O35" s="66"/>
       <c r="P35" s="66"/>
       <c r="Q35" s="66"/>
-      <c r="R35" s="74"/>
-      <c r="S35" s="74"/>
-      <c r="T35" s="74"/>
-      <c r="U35" s="74"/>
-      <c r="V35" s="74"/>
-      <c r="W35" s="74"/>
-      <c r="X35" s="74"/>
-      <c r="Y35" s="74"/>
-      <c r="Z35" s="74"/>
-      <c r="AA35" s="74"/>
-      <c r="AB35" s="74"/>
-      <c r="AC35" s="74"/>
-      <c r="AD35" s="75"/>
-      <c r="AE35" s="76"/>
-      <c r="AF35" s="76"/>
-      <c r="AG35" s="76"/>
-      <c r="AH35" s="76"/>
-      <c r="AI35" s="77"/>
+      <c r="R35" s="73"/>
+      <c r="S35" s="73"/>
+      <c r="T35" s="73"/>
+      <c r="U35" s="73"/>
+      <c r="V35" s="73"/>
+      <c r="W35" s="73"/>
+      <c r="X35" s="73"/>
+      <c r="Y35" s="73"/>
+      <c r="Z35" s="73"/>
+      <c r="AA35" s="73"/>
+      <c r="AB35" s="73"/>
+      <c r="AC35" s="73"/>
+      <c r="AD35" s="74"/>
+      <c r="AE35" s="75"/>
+      <c r="AF35" s="75"/>
+      <c r="AG35" s="75"/>
+      <c r="AH35" s="75"/>
+      <c r="AI35" s="76"/>
       <c r="AJ35" s="8"/>
     </row>
     <row r="36" spans="2:36" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -3545,24 +3420,24 @@
       <c r="O36" s="66"/>
       <c r="P36" s="66"/>
       <c r="Q36" s="66"/>
-      <c r="R36" s="74"/>
-      <c r="S36" s="74"/>
-      <c r="T36" s="74"/>
-      <c r="U36" s="74"/>
-      <c r="V36" s="74"/>
-      <c r="W36" s="74"/>
-      <c r="X36" s="74"/>
-      <c r="Y36" s="74"/>
-      <c r="Z36" s="74"/>
-      <c r="AA36" s="74"/>
-      <c r="AB36" s="74"/>
-      <c r="AC36" s="74"/>
-      <c r="AD36" s="75"/>
-      <c r="AE36" s="76"/>
-      <c r="AF36" s="76"/>
-      <c r="AG36" s="76"/>
-      <c r="AH36" s="76"/>
-      <c r="AI36" s="77"/>
+      <c r="R36" s="73"/>
+      <c r="S36" s="73"/>
+      <c r="T36" s="73"/>
+      <c r="U36" s="73"/>
+      <c r="V36" s="73"/>
+      <c r="W36" s="73"/>
+      <c r="X36" s="73"/>
+      <c r="Y36" s="73"/>
+      <c r="Z36" s="73"/>
+      <c r="AA36" s="73"/>
+      <c r="AB36" s="73"/>
+      <c r="AC36" s="73"/>
+      <c r="AD36" s="74"/>
+      <c r="AE36" s="75"/>
+      <c r="AF36" s="75"/>
+      <c r="AG36" s="75"/>
+      <c r="AH36" s="75"/>
+      <c r="AI36" s="76"/>
       <c r="AJ36" s="8"/>
     </row>
     <row r="37" spans="2:36" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -4464,13 +4339,13 @@
     </row>
     <row r="68" spans="2:36" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B68" s="17"/>
-      <c r="C68" s="73" t="s">
+      <c r="C68" s="77" t="s">
         <v>51</v>
       </c>
-      <c r="D68" s="73"/>
-      <c r="E68" s="73"/>
-      <c r="F68" s="73"/>
-      <c r="G68" s="73"/>
+      <c r="D68" s="77"/>
+      <c r="E68" s="77"/>
+      <c r="F68" s="77"/>
+      <c r="G68" s="77"/>
       <c r="H68" s="55" t="s">
         <v>52</v>
       </c>
@@ -4486,13 +4361,13 @@
       <c r="P68" s="71"/>
       <c r="Q68" s="71"/>
       <c r="R68" s="72"/>
-      <c r="S68" s="73" t="s">
+      <c r="S68" s="77" t="s">
         <v>54</v>
       </c>
-      <c r="T68" s="73"/>
-      <c r="U68" s="73"/>
-      <c r="V68" s="73"/>
-      <c r="W68" s="73"/>
+      <c r="T68" s="77"/>
+      <c r="U68" s="77"/>
+      <c r="V68" s="77"/>
+      <c r="W68" s="77"/>
       <c r="X68" s="100"/>
       <c r="Y68" s="100"/>
       <c r="Z68" s="100"/>

</xml_diff>